<commit_message>
feat: add Emag API response and product interfaces
- Introduced EmagApiResponse interface for handling API responses.
- Added EmagStockValue and EmagHandlingTimeValue interfaces for stock and handling time data.
- Created EmagProduct and EmagProductOfferPayload interfaces for product details and offers.
- Defined EmagProductMeasurementPayload for product measurements.
- Added EmagOffer interface for managing offers.
- Introduced EmagStockUpdate and EmagPriceUpdate interfaces for stock and price updates.
- Created EmagOrder and EmagOrderProduct interfaces for order management.
- Added EmagWebhookEvent interface for handling webhook events.
</commit_message>
<xml_diff>
--- a/Beok_products_Prices 2026.xlsx
+++ b/Beok_products_Prices 2026.xlsx
@@ -1,31 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\H588238\Downloads\My Documents\02 BEOK BG\1st order\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\H588238\Downloads\My Documents\VS CODE\BEOKBG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975E1630-807C-4534-A78F-279E3E8AF99C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83837FA2-D994-48BA-B033-2A391278856B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Prices" sheetId="1" r:id="rId1"/>
+    <sheet name="emag_overrides" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
   <si>
     <t>TGM50-WIFI-EP</t>
   </si>
@@ -106,16 +118,41 @@
   </si>
   <si>
     <t>Total Profit</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>BEOK</t>
+  </si>
+  <si>
+    <t>EAN</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>width</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>length</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
+    <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -130,8 +167,16 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -144,8 +189,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -238,11 +295,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -281,11 +358,453 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="169" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFE6E6E6"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFE6E6E6"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFE6E6E6"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFE6E6E6"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -750,20 +1269,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD8E6B6D-1DD3-4F0C-86B9-BE7A319FFBE5}" name="Table1" displayName="Table1" ref="A1:K17" totalsRowShown="0" dataDxfId="13" headerRowBorderDxfId="14" tableBorderDxfId="12" totalsRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD8E6B6D-1DD3-4F0C-86B9-BE7A319FFBE5}" name="Table1" displayName="Table1" ref="A1:K17" totalsRowShown="0" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26" totalsRowBorderDxfId="25">
   <autoFilter ref="A1:K17" xr:uid="{CD8E6B6D-1DD3-4F0C-86B9-BE7A319FFBE5}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{07B2CB3F-FB12-4FFE-B29F-80C78129A0B3}" name="Model" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{2C19763C-CE3D-4556-A0B2-F62D3EA135D2}" name="Qty" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{014512B3-03D0-4636-853B-9164AE73A960}" name="Factory Price (USD)" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{54A37127-B297-404F-B260-6EBF7B328562}" name="Landed Cost (EUR incl. shipping)" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{5C977046-589B-471B-87F7-A65DC3ABF4E7}" name="Competitor Amazon Price (incl. VAT)" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{DE844D21-D3FF-4927-ACDC-46496E1EC5FF}" name="Net Price (excl. VAT)" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{0CB03D02-817C-4F9C-A8C7-B92ED2469668}" name="eMAG Fee (12%)" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{60C8B842-26DA-402F-9209-B222E2DEE319}" name="Other Costs" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{47EBA81C-A220-4873-8AA6-479ED412FDF9}" name="Profit per Unit" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{9147229C-EB3E-40AE-8E48-1D8422C012AD}" name="Margin" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{1031A2C4-C9EA-40BE-845A-F1898E1FA41E}" name="Total Profit" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{07B2CB3F-FB12-4FFE-B29F-80C78129A0B3}" name="Model" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{2C19763C-CE3D-4556-A0B2-F62D3EA135D2}" name="Qty" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{014512B3-03D0-4636-853B-9164AE73A960}" name="Factory Price (USD)" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{54A37127-B297-404F-B260-6EBF7B328562}" name="Landed Cost (EUR incl. shipping)" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{5C977046-589B-471B-87F7-A65DC3ABF4E7}" name="Competitor Amazon Price (incl. VAT)" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{DE844D21-D3FF-4927-ACDC-46496E1EC5FF}" name="Net Price (excl. VAT)" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{0CB03D02-817C-4F9C-A8C7-B92ED2469668}" name="eMAG Fee (12%)" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{60C8B842-26DA-402F-9209-B222E2DEE319}" name="Other Costs" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{47EBA81C-A220-4873-8AA6-479ED412FDF9}" name="Profit per Unit" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{9147229C-EB3E-40AE-8E48-1D8422C012AD}" name="Margin" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{1031A2C4-C9EA-40BE-845A-F1898E1FA41E}" name="Total Profit" dataDxfId="14"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7B277A1C-2E67-4613-B61E-3DD01663EB5D}" name="Table2" displayName="Table2" ref="A1:I17" totalsRowShown="0" headerRowDxfId="8" dataDxfId="9" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+  <autoFilter ref="A1:I17" xr:uid="{7B277A1C-2E67-4613-B61E-3DD01663EB5D}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{FA3A1C50-58BF-48EF-9CD1-CE1979D2B0AE}" name="Brand" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{32B518C0-4810-473E-ABAC-3261CBDDB365}" name="Model" dataDxfId="7">
+      <calculatedColumnFormula>Table1[[#This Row],[Model]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{272EAB41-8E38-4F89-A138-E3166B1D801B}" name="Qty" dataDxfId="6">
+      <calculatedColumnFormula>Table1[[#This Row],[Qty]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{E14DE9B2-1346-41DC-B48C-057BBE02E423}" name="EAN" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{B35EC088-2A82-4A0F-A2E6-DB8E54A0CC1C}" name="Description" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{9B067A65-755F-4043-B9AA-E666E5C8597F}" name="weight" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{9DEEA8CF-68BD-46CE-A1B5-FAD1590D7ECC}" name="width" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{439009A2-D751-47DA-BF7B-1C26886DFA2D}" name="height" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{FAF760A8-F4B6-4246-991D-ECADF9741398}" name="length" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1651,6 +2192,409 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2116AC5B-3745-442C-9DF5-DC5E9A22AF4E}">
+  <dimension ref="A1:I36"/>
+  <sheetFormatPr defaultColWidth="20.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="16" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TGM50-WIFI-EP</v>
+      </c>
+      <c r="C2" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+    </row>
+    <row r="3" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TGM50-WIFI-WP</v>
+      </c>
+      <c r="C3" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+    </row>
+    <row r="4" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TGM50B-WIFI-EP</v>
+      </c>
+      <c r="C4" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+    </row>
+    <row r="5" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TGM50B-WIFI-WP</v>
+      </c>
+      <c r="C5" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+    </row>
+    <row r="6" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TCC31-WIFI-EP</v>
+      </c>
+      <c r="C6" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+    </row>
+    <row r="7" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TCC31-WIFI-WP</v>
+      </c>
+      <c r="C7" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+    </row>
+    <row r="8" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TGR85-WIFI-WPB</v>
+      </c>
+      <c r="C8" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+    </row>
+    <row r="9" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TCC31-WIFI-WPB</v>
+      </c>
+      <c r="C9" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+    </row>
+    <row r="10" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>BOT-R7W-X-WIFI</v>
+      </c>
+      <c r="C10" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+    </row>
+    <row r="11" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>BOT-R7B-X-WIFI</v>
+      </c>
+      <c r="C11" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+    </row>
+    <row r="12" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>BOT-R8X-WIFI</v>
+      </c>
+      <c r="C12" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>20</v>
+      </c>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+    </row>
+    <row r="13" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TRV-604</v>
+      </c>
+      <c r="C13" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>40</v>
+      </c>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+    </row>
+    <row r="14" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>TRV-705WF</v>
+      </c>
+      <c r="C14" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>40</v>
+      </c>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+    </row>
+    <row r="15" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>CCT-28-X</v>
+      </c>
+      <c r="C15" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>10</v>
+      </c>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+    </row>
+    <row r="16" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="15" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>BOT-R7X-WIFI-NR</v>
+      </c>
+      <c r="C16" s="20">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>40</v>
+      </c>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+    </row>
+    <row r="17" spans="1:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <f>Table1[[#This Row],[Model]]</f>
+        <v>RZ-D01.230-NC</v>
+      </c>
+      <c r="C17" s="21">
+        <f>Table1[[#This Row],[Qty]]</f>
+        <v>40</v>
+      </c>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+    </row>
+    <row r="22" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F22" s="14"/>
+    </row>
+    <row r="23" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F23" s="14"/>
+    </row>
+    <row r="24" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F24" s="14"/>
+    </row>
+    <row r="25" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F25" s="14"/>
+    </row>
+    <row r="26" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F26" s="14"/>
+    </row>
+    <row r="27" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F27" s="14"/>
+    </row>
+    <row r="28" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F28" s="14"/>
+    </row>
+    <row r="29" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F29" s="14"/>
+    </row>
+    <row r="30" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F30" s="14"/>
+    </row>
+    <row r="31" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F31" s="14"/>
+    </row>
+    <row r="32" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F32" s="14"/>
+    </row>
+    <row r="33" spans="6:6" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F33" s="14"/>
+    </row>
+    <row r="34" spans="6:6" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F34" s="14"/>
+    </row>
+    <row r="35" spans="6:6" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F35" s="14"/>
+    </row>
+    <row r="36" spans="6:6" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="F36" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{d546e5e1-5d42-4630-bacd-c69bfdcbd5e8}" enabled="1" method="Standard" siteId="{96ece526-9c7d-48b0-8daf-8b93c90a5d18}" contentBits="0" removed="0"/>

</xml_diff>